<commit_message>
nuevos campos db Order
</commit_message>
<xml_diff>
--- a/db/orden.xlsx
+++ b/db/orden.xlsx
@@ -8,19 +8,30 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Lyle\Pulloc\Project\gestor-restaurante\db\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC2F2253-362D-40D9-BB67-77AE20328908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{916E3720-0D75-4C40-98CD-1E4170073AEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Uid</t>
   </si>
@@ -41,6 +52,15 @@
   </si>
   <si>
     <t>[{"Producto": {"Uid": "1", "Name": "Pizza", "Image": "[\"pizza.jpg\"]", "Price": 30000, "Discount_price": 25000, "IsActive": true, "Description": "Pizza familiar", "Items": "[{\"Name\": \"Queso\", \"amount\": \"1\"}, {\"Name\": \"Jam\\u00f3n\", \"amount\": \"2\"}]"}, "amount": 2, "additional_information": "Sin cebolla"}]</t>
+  </si>
+  <si>
+    <t>Fecha</t>
+  </si>
+  <si>
+    <t>Hora</t>
+  </si>
+  <si>
+    <t>Mesero</t>
   </si>
 </sst>
 </file>
@@ -72,7 +92,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -95,15 +115,30 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -442,10 +477,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="6" max="6" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -458,8 +497,17 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -471,6 +519,15 @@
       </c>
       <c r="D2" t="s">
         <v>6</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2" s="3">
+        <v>45810</v>
+      </c>
+      <c r="G2">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
buscador erroneo en orden
</commit_message>
<xml_diff>
--- a/db/orden.xlsx
+++ b/db/orden.xlsx
@@ -1,41 +1,62 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Lyle\Pulloc\Project\gestor-restaurante\db\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74045335-44F9-4A96-886C-E697BB23BE0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="5115" yWindow="3075" windowWidth="15375" windowHeight="7995" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="ordenes" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="10">
+  <si>
+    <t>Uid</t>
+  </si>
+  <si>
+    <t>table</t>
+  </si>
+  <si>
+    <t>Description_general</t>
+  </si>
+  <si>
+    <t>Orders_group</t>
+  </si>
+  <si>
+    <t>Mesero</t>
+  </si>
+  <si>
+    <t>Fecha</t>
+  </si>
+  <si>
+    <t>Hora</t>
+  </si>
+  <si>
+    <t>Mesa familiar</t>
+  </si>
+  <si>
+    <t>[{"Producto": {"Uid": "1", "Name": "Pizza", "Image": "[\"pizza.jpg\"]", "Price": 30000, "Discount_price": 25000, "IsActive": true, "Description": "Pizza familiar", "Items": "[{\"Name\": \"Queso\", \"amount\": \"1\"}, {\"Name\": \"Jam\\u00f3n\", \"amount\": \"2\"}]"}, "amount": 2, "additional_information": "Sin cebolla"}]</t>
+  </si>
+  <si>
+    <t>Mesa sola</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -72,6 +93,14 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,44 +425,45 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Uid</v>
-      </c>
-      <c r="B1" t="str">
-        <v>table</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Description_general</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Orders_group</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Mesero</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Fecha</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Hora</v>
+    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2">
         <v>3</v>
       </c>
-      <c r="C2" t="str">
-        <v>Mesa familiar</v>
-      </c>
-      <c r="D2" t="str">
-        <v>[{"Producto": {"Uid": "1", "Name": "Pizza", "Image": "[\"pizza.jpg\"]", "Price": 30000, "Discount_price": 25000, "IsActive": true, "Description": "Pizza familiar", "Items": "[{\"Name\": \"Queso\", \"amount\": \"1\"}, {\"Name\": \"Jam\\u00f3n\", \"amount\": \"2\"}]"}, "amount": 2, "additional_information": "Sin cebolla"}]</v>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -445,9 +475,79 @@
         <v>18</v>
       </c>
     </row>
+    <row r="3" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>45810</v>
+      </c>
+      <c r="G3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>45810</v>
+      </c>
+      <c r="G4">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>45810</v>
+      </c>
+      <c r="G5">
+        <v>18</v>
+      </c>
+    </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+    <ignoredError sqref="A1:G1 B2:G2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Arreglo de codigo, y buscador agregado en Orden
</commit_message>
<xml_diff>
--- a/db/orden.xlsx
+++ b/db/orden.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Lyle\Pulloc\Project\gestor-restaurante\db\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74045335-44F9-4A96-886C-E697BB23BE0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89971613-ED6D-4EC6-B47E-0A3BEEB3770A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5115" yWindow="3075" windowWidth="15375" windowHeight="7995" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -427,9 +427,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -452,7 +452,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -475,12 +475,12 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C3" t="s">
         <v>9</v>
@@ -498,12 +498,12 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C4" t="s">
         <v>9</v>
@@ -521,7 +521,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>

</xml_diff>